<commit_message>
Secure Snowflake credentials and update unit testing framework
</commit_message>
<xml_diff>
--- a/user/input/ut_input.xlsx
+++ b/user/input/ut_input.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="28">
   <si>
     <t>TC001</t>
   </si>
@@ -60,9 +60,6 @@
     <t>Test_case_type</t>
   </si>
   <si>
-    <t>Source_table</t>
-  </si>
-  <si>
     <t>Target_table</t>
   </si>
   <si>
@@ -94,9 +91,6 @@
   </si>
   <si>
     <t>special_character_validation</t>
-  </si>
-  <si>
-    <t>bronze_customers_delta</t>
   </si>
   <si>
     <t>silver_customers_delta</t>
@@ -440,19 +434,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="16.81640625" customWidth="1"/>
     <col min="2" max="2" width="26.81640625" customWidth="1"/>
-    <col min="3" max="3" width="22.26953125" customWidth="1"/>
-    <col min="4" max="4" width="21.54296875" customWidth="1"/>
-    <col min="5" max="5" width="17.1796875" customWidth="1"/>
-    <col min="6" max="6" width="19.08984375" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
+    <col min="3" max="3" width="21.54296875" customWidth="1"/>
+    <col min="4" max="4" width="17.1796875" customWidth="1"/>
+    <col min="5" max="5" width="19.08984375" customWidth="1"/>
+    <col min="6" max="6" width="13.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -463,198 +456,162 @@
         <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="E1" s="1"/>
       <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" spans="1:7">
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
         <v>26</v>
       </c>
-      <c r="D11" t="s">
+      <c r="B12" t="s">
         <v>27</v>
       </c>
-      <c r="E11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" t="s">
-        <v>29</v>
-      </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>